<commit_message>
Tracker: journal, questions and chat rows updated 2026-09-11
Mobile rows 35 and 36 to testing, 47 chat in progress, with dated evidence notes; web rows 129 and 130 notes.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/МнКардио_тендерийн_ажлын_жагсаалт.xlsx
+++ b/МнКардио_тендерийн_ажлын_жагсаалт.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2129" uniqueCount="748">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2130" uniqueCount="749">
   <si>
     <t>ХЯНАЛТЫН САМБАР</t>
   </si>
@@ -772,10 +772,10 @@
     <t>Гар утасны аппликэйшнд зориулсан API нээх — хөгжүүлэлт, тохиргоо</t>
   </si>
   <si>
-    <t>2026-09-10: Гар утасны API нээгдэв — /api/doctor (12 маршрут: /me, /visits, /monitoring, /advice, /reports/summary, /patients) ба /api/patient (16 маршрут: /me, /journal, /questions, /advice, /risk, /evisits, /rehab/*), server.js:373-382. Бодит HTTP төлөвийн код, жижиг үсгийн {success,message,data} бүрхүүлтэй. Гэрээний бүрэн тодорхойлолт: mobile/API.md.</t>
-  </si>
-  <si>
-    <t>2026-09-10: /api/doctor ба /api/patient давхаргыг tests/acceptance харвалтаар туршив (248 маршрут дуудагдав, 48 бичих урсгал). Гар утасны клиент бичигдээгүй тул төгсгөл-төгсгөлийн интеграц дуусаагүй.</t>
+    <t>2026-09-10: Гар утасны API нээгдэв — /api/doctor (12 маршрут: /me, /visits, /monitoring, /advice, /reports/summary, /patients) ба /api/patient (16 маршрут: /me, /journal, /questions, /advice, /risk, /evisits, /rehab/*), server.js:373-382. Бодит HTTP төлөвийн код, жижиг үсгийн {success,message,data} бүрхүүлтэй. Гэрээний бүрэн тодорхойлолт: mobile/API.md. | 2026-09-11: /api/doctor-д 2 маршрут нэмэгдэв — GET|POST /monitoring/:patientId/questions (эмч асуултад хариулах). /api/patient/journal ба /questions бичилт засагдав (83bc3c0).</t>
+  </si>
+  <si>
+    <t>2026-09-10: /api/doctor ба /api/patient давхаргыг tests/acceptance харвалтаар туршив (248 маршрут дуудагдав, 48 бичих урсгал). Гар утасны клиент бичигдээгүй тул төгсгөл-төгсгөлийн интеграц дуусаагүй. | 2026-09-11: Гар утасны клиент mobile/app-д бий (165ce3c) — "клиент бичигдээгүй" гэсэн өмнөх тэмдэглэл хуучирсан. Тест орчинд тэмдэглэл, асуулт–хариулт, чат (үйлчлүүлэгч→эмч) урсгалыг серверийн түвшинд төгсгөл хүртэл шалгав; клиентийн засварууд mobile/CHAT-CLIENT-FIXES.md.</t>
   </si>
   <si>
     <t>Тест, чанарын баталгаажуулалт</t>
@@ -1399,7 +1399,7 @@
     <t>Өдөр тутмын бүртгэл орж, график хэлбэрээр харагдана</t>
   </si>
   <si>
-    <t>2026-09-10: Энэ дэлгэцийг тэжээх сервер тал бэлэн — GET|POST /api/patient/journal, /journal/summary (веб жагсаалтын мөр #129). Гар утасны апп-ын код бичигдээгүй тул гүйцэтгэл 0 хэвээр.</t>
+    <t>2026-09-10: Энэ дэлгэцийг тэжээх сервер тал бэлэн — GET|POST /api/patient/journal, /journal/summary (веб жагсаалтын мөр #129). Гар утасны апп-ын код бичигдээгүй тул гүйцэтгэл 0 хэвээр. | 2026-09-11: Тэмдэглэл хадгалах POST /api/patient/journal бүх оролдлогод 500 өгдөг байсныг засав — rec_status 'A' int баганад бичигдэж, id/id_group/user_mod/date_modif хоосон үлддэг байв; BaseCreate руу шилжүүлэв (commit 83bc3c0). Тест орчинд хадгалах, жагсаалтад харах бодитоор шалгагдав. Гар утасны дэлгэц mobile/app-д бий (165ce3c); төхөөрөмж дээр бид ажиллуулж шалгаагүй.</t>
   </si>
   <si>
     <t>2.3 Эмчээс асуух асуулт</t>
@@ -1411,7 +1411,7 @@
     <t>Асуулт илгээгдэж, эмчид хүрнэ</t>
   </si>
   <si>
-    <t>2026-09-10: Энэ дэлгэцийг тэжээх сервер тал бэлэн — GET|POST /api/patient/questions (веб жагсаалтын мөр #129). Гар утасны апп-ын код бичигдээгүй тул гүйцэтгэл 0 хэвээр.</t>
+    <t>2026-09-10: Энэ дэлгэцийг тэжээх сервер тал бэлэн — GET|POST /api/patient/questions (веб жагсаалтын мөр #129). Гар утасны апп-ын код бичигдээгүй тул гүйцэтгэл 0 хэвээр. | 2026-09-11: Асуулт илгээх POST /api/patient/questions 500 өгдөг байсныг засав (ижил шалтгаан, 83bc3c0). Эмч хариулах GET|POST /api/doctor/monitoring/:patientId/questions нэмэгдэв (mobile/API.md §29). Тест орчинд асуулт → эмчийн хариу → үйлчлүүлэгч эмчийн нэртэй хариугаа харах урсгал бодитоор шалгагдав. Гар утасны дэлгэц mobile/app-д бий; эмчийн модульд асуулт харах дэлгэц хараахан байхгүй (mobile/CHAT-CLIENT-FIXES.md §6).</t>
   </si>
   <si>
     <t>2.4 Эмчийн зөвлөгөө</t>
@@ -1526,6 +1526,9 @@
   </si>
   <si>
     <t>Эмч, үйлчлүүлэгч хооронд бодит цагийн харилцаа</t>
+  </si>
+  <si>
+    <t>2026-09-11: Сервер: үйлчлүүлэгч өөрийг нь хяналтад авсан эмчтэй чатлах боломжтой болов — өмнө нь зөвхөн эмчийн баг тооцогдож, тест DB-д үйлчлүүлэгчийн бичсэн мессеж 0 байв; тест орчинд StartChat амжилттай. Вэб: эмч асуултын цонхноос ("Чатаар бичих") үйлчлүүлэгчтэй чат эхлүүлэх товч нэмэгдэж, тест орчинд хөтөч дээр шалгав (MonitorQuestion.jsx). Гар утасны клиентийн чатын алдаанууд (давхар бөмбөлөг, токен дуусахад socket зогсох, татгалзал чимээгүй, "бичиж байна", хавсралт) mobile/CHAT-CLIENT-FIXES.md-д хөгжүүлэгчид шилжүүлэв.</t>
   </si>
   <si>
     <t>Мэдэгдэл (Notification)</t>
@@ -10725,849 +10728,849 @@
       </c>
       <c r="L157" s="19"/>
     </row>
-    <row r="158" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="159" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="160" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="161" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="162" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="163" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="164" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="165" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="166" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="167" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="168" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="169" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="170" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="171" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="172" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="173" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="174" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="175" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="176" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="177" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="178" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="179" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="180" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="181" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="182" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="183" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="184" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="185" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="186" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="187" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="188" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="189" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="190" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="191" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="192" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="193" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="194" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="195" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="196" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="197" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="198" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="199" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="200" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="201" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="202" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="203" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="204" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="205" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="206" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="207" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="208" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="209" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="210" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="211" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="212" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="213" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="214" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="215" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="216" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="217" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="218" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="219" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="220" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="221" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="222" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="223" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="224" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="225" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="226" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="227" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="228" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="229" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="230" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="231" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="232" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="233" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="234" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="235" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="236" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="237" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="238" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="239" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="240" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="241" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="242" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="243" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="244" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="245" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="246" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="247" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="248" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="249" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="250" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="251" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="252" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="253" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="254" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="255" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="256" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="257" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="258" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="259" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="260" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="261" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="262" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="263" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="264" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="265" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="266" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="267" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="268" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="269" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="270" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="271" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="272" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="273" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="274" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="275" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="276" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="277" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="278" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="279" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="280" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="281" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="282" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="283" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="284" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="285" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="286" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="287" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="288" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="289" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="290" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="291" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="292" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="293" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="294" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="295" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="296" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="297" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="298" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="299" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="300" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="301" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="302" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="303" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="304" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="305" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="306" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="307" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="308" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="309" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="310" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="311" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="312" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="313" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="314" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="315" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="316" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="317" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="318" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="319" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="320" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="321" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="322" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="323" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="324" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="325" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="326" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="327" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="328" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="329" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="330" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="331" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="332" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="333" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="334" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="335" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="336" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="337" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="338" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="339" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="340" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="341" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="342" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="343" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="344" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="345" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="346" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="347" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="348" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="349" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="350" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="351" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="352" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="353" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="354" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="355" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="356" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="357" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="358" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="359" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="360" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="361" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="362" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="363" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="364" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="365" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="366" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="367" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="368" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="369" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="370" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="371" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="372" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="373" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="374" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="375" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="376" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="377" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="378" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="379" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="380" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="381" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="382" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="383" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="384" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="385" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="386" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="387" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="388" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="389" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="390" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="391" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="392" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="393" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="394" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="395" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="396" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="397" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="398" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="399" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="400" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="401" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="402" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="403" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="404" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="405" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="406" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="407" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="408" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="409" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="410" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="411" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="412" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="413" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="414" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="415" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="416" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="417" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="418" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="419" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="420" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="421" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="422" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="423" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="424" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="425" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="426" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="427" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="428" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="429" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="430" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="431" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="432" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="433" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="434" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="435" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="436" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="437" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="438" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="439" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="440" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="441" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="442" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="443" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="444" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="445" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="446" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="447" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="448" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="449" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="450" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="451" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="452" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="453" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="454" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="455" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="456" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="457" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="458" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="459" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="460" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="461" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="462" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="463" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="464" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="465" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="466" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="467" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="468" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="469" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="470" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="471" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="472" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="473" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="474" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="475" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="476" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="477" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="478" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="479" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="480" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="481" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="482" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="483" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="484" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="485" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="486" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="487" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="488" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="489" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="490" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="491" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="492" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="493" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="494" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="495" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="496" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="497" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="498" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="499" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="500" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="501" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="502" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="503" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="504" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="505" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="506" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="507" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="508" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="509" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="510" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="511" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="512" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="513" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="514" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="515" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="516" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="517" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="518" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="519" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="520" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="521" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="522" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="523" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="524" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="525" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="526" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="527" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="528" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="529" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="530" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="531" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="532" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="533" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="534" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="535" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="536" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="537" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="538" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="539" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="540" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="541" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="542" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="543" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="544" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="545" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="546" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="547" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="548" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="549" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="550" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="551" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="552" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="553" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="554" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="555" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="556" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="557" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="558" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="559" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="560" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="561" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="562" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="563" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="564" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="565" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="566" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="567" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="568" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="569" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="570" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="571" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="572" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="573" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="574" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="575" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="576" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="577" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="578" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="579" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="580" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="581" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="582" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="583" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="584" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="585" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="586" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="587" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="588" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="589" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="590" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="591" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="592" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="593" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="594" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="595" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="596" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="597" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="598" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="599" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="600" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="601" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="602" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="603" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="604" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="605" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="606" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="607" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="608" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="609" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="610" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="611" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="612" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="613" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="614" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="615" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="616" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="617" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="618" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="619" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="620" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="621" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="622" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="623" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="624" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="625" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="626" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="627" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="628" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="629" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="630" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="631" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="632" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="633" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="634" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="635" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="636" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="637" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="638" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="639" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="640" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="641" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="642" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="643" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="644" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="645" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="646" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="647" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="648" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="649" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="650" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="651" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="652" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="653" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="654" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="655" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="656" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="657" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="658" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="659" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="660" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="661" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="662" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="663" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="664" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="665" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="666" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="667" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="668" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="669" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="670" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="671" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="672" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="673" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="674" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="675" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="676" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="677" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="678" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="679" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="680" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="681" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="682" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="683" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="684" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="685" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="686" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="687" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="688" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="689" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="690" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="691" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="692" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="693" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="694" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="695" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="696" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="697" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="698" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="699" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="700" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="701" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="702" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="703" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="704" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="705" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="706" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="707" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="708" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="709" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="710" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="711" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="712" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="713" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="714" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="715" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="716" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="717" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="718" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="719" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="720" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="721" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="722" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="723" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="724" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="725" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="726" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="727" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="728" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="729" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="730" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="731" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="732" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="733" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="734" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="735" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="736" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="737" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="738" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="739" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="740" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="741" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="742" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="743" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="744" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="745" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="746" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="747" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="748" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="749" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="750" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="751" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="752" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="753" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="754" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="755" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="756" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="757" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="758" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="759" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="760" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="761" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="762" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="763" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="764" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="765" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="766" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="767" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="768" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="769" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="770" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="771" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="772" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="773" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="774" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="775" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="776" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="777" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="778" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="779" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="780" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="781" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="782" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="783" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="784" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="785" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="786" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="787" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="788" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="789" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="790" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="791" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="792" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="793" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="794" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="795" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="796" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="797" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="798" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="799" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="800" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="801" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="802" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="803" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="804" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="805" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="806" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="807" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="808" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="809" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="810" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="811" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="812" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="813" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="814" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="815" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="816" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="817" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="818" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="819" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="820" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="821" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="822" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="823" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="824" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="825" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="826" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="827" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="828" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="829" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="830" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="831" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="832" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="833" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="834" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="835" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="836" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="837" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="838" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="839" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="840" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="841" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="842" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="843" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="844" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="845" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="846" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="847" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="848" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="849" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="850" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="851" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="852" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="853" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="854" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="855" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="856" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="857" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="858" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="859" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="860" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="861" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="862" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="863" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="864" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="865" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="866" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="867" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="868" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="869" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="870" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="871" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="872" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="873" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="874" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="875" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="876" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="877" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="878" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="879" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="880" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="881" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="882" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="883" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="884" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="885" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="886" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="887" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="888" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="889" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="890" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="891" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="892" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="893" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="894" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="895" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="896" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="897" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="898" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="899" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="900" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="901" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="902" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="903" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="904" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="905" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="906" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="907" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="908" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="909" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="910" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="911" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="912" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="913" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="914" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="915" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="916" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="917" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="918" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="919" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="920" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="921" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="922" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="923" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="924" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="925" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="926" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="927" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="928" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="929" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="930" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="931" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="932" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="933" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="934" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="935" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="936" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="937" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="938" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="939" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="940" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="941" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="942" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="943" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="944" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="945" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="946" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="947" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="948" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="949" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="950" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="951" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="952" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="953" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="954" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="955" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="956" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="957" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="958" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="959" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="960" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="961" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="962" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="963" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="964" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="965" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="966" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="967" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="968" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="969" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="970" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="971" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="972" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="973" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="974" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="975" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="976" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="977" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="978" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="979" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="980" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="981" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="982" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="983" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="984" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="985" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="986" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="987" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="988" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="989" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="990" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="991" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="992" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="993" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="994" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="995" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="996" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="997" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="998" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="999" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="1000" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25"/>
+    <row r="158" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="159" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="160" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="161" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="162" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="163" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="164" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="165" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="166" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="167" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="168" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="169" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="170" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="171" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="172" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="173" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="174" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="175" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="176" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="180" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="181" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="182" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="183" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="184" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="185" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="186" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="187" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="188" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="189" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="190" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="191" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="192" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="193" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="194" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="195" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="196" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="197" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="198" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="199" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="200" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="201" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="202" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A4:L157"/>
   <conditionalFormatting sqref="H5:H157">
@@ -11635,7 +11638,7 @@
     <col min="13" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>38</v>
       </c>
@@ -12978,10 +12981,10 @@
         <v>46255</v>
       </c>
       <c r="I39" s="17" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J39" s="23">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K39" s="19" t="s">
         <v>458</v>
@@ -13016,10 +13019,10 @@
         <v>46256</v>
       </c>
       <c r="I40" s="17" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J40" s="23">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K40" s="19" t="s">
         <v>462</v>
@@ -13424,15 +13427,17 @@
         <v>46267</v>
       </c>
       <c r="I51" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J51" s="23">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K51" s="19" t="s">
         <v>501</v>
       </c>
-      <c r="L51" s="19"/>
+      <c r="L51" s="19" t="s">
+        <v>502</v>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="17">
@@ -13445,10 +13450,10 @@
         <v>498</v>
       </c>
       <c r="D52" s="19" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="E52" s="19" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F52" s="17" t="s">
         <v>16</v>
@@ -13466,7 +13471,7 @@
         <v>0</v>
       </c>
       <c r="K52" s="19" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="L52" s="19"/>
     </row>
@@ -13481,10 +13486,10 @@
         <v>498</v>
       </c>
       <c r="D53" s="19" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E53" s="19" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F53" s="17" t="s">
         <v>16</v>
@@ -13502,7 +13507,7 @@
         <v>0</v>
       </c>
       <c r="K53" s="19" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="L53" s="19"/>
     </row>
@@ -13514,13 +13519,13 @@
         <v>49</v>
       </c>
       <c r="C54" s="19" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D54" s="19" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E54" s="19" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="F54" s="17" t="s">
         <v>16</v>
@@ -13538,10 +13543,10 @@
         <v>0</v>
       </c>
       <c r="K54" s="19" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="L54" s="19" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -13552,13 +13557,13 @@
         <v>49</v>
       </c>
       <c r="C55" s="19" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D55" s="19" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="E55" s="19" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="F55" s="17" t="s">
         <v>16</v>
@@ -13576,10 +13581,10 @@
         <v>0</v>
       </c>
       <c r="K55" s="19" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="L55" s="19" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -13590,13 +13595,13 @@
         <v>49</v>
       </c>
       <c r="C56" s="19" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D56" s="19" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E56" s="19" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F56" s="17" t="s">
         <v>16</v>
@@ -13614,7 +13619,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="19" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="L56" s="19"/>
     </row>
@@ -13626,13 +13631,13 @@
         <v>49</v>
       </c>
       <c r="C57" s="19" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D57" s="19" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="E57" s="19" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="F57" s="17" t="s">
         <v>16</v>
@@ -13650,10 +13655,10 @@
         <v>0</v>
       </c>
       <c r="K57" s="19" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="L57" s="19" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -13664,13 +13669,13 @@
         <v>49</v>
       </c>
       <c r="C58" s="19" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D58" s="19" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="E58" s="19" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F58" s="17" t="s">
         <v>17</v>
@@ -13688,10 +13693,10 @@
         <v>0</v>
       </c>
       <c r="K58" s="19" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="L58" s="19" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -13702,13 +13707,13 @@
         <v>49</v>
       </c>
       <c r="C59" s="19" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D59" s="19" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E59" s="19" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F59" s="17" t="s">
         <v>16</v>
@@ -13726,10 +13731,10 @@
         <v>0</v>
       </c>
       <c r="K59" s="19" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="L59" s="19" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -13740,13 +13745,13 @@
         <v>49</v>
       </c>
       <c r="C60" s="19" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D60" s="19" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="E60" s="19" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="F60" s="17" t="s">
         <v>16</v>
@@ -13764,10 +13769,10 @@
         <v>0</v>
       </c>
       <c r="K60" s="19" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="L60" s="19" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -13778,13 +13783,13 @@
         <v>51</v>
       </c>
       <c r="C61" s="19" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D61" s="19" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E61" s="19" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F61" s="17" t="s">
         <v>16</v>
@@ -13802,7 +13807,7 @@
         <v>0</v>
       </c>
       <c r="K61" s="19" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="L61" s="19"/>
     </row>
@@ -13814,13 +13819,13 @@
         <v>51</v>
       </c>
       <c r="C62" s="19" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D62" s="19" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="E62" s="19" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="F62" s="17" t="s">
         <v>16</v>
@@ -13838,7 +13843,7 @@
         <v>0</v>
       </c>
       <c r="K62" s="19" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="L62" s="19"/>
     </row>
@@ -13850,13 +13855,13 @@
         <v>51</v>
       </c>
       <c r="C63" s="19" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D63" s="19" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E63" s="19" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F63" s="17" t="s">
         <v>17</v>
@@ -13874,7 +13879,7 @@
         <v>0</v>
       </c>
       <c r="K63" s="19" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="L63" s="19"/>
     </row>
@@ -13886,13 +13891,13 @@
         <v>51</v>
       </c>
       <c r="C64" s="19" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D64" s="19" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="E64" s="19" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="F64" s="17" t="s">
         <v>16</v>
@@ -13910,7 +13915,7 @@
         <v>0</v>
       </c>
       <c r="K64" s="19" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="L64" s="19"/>
     </row>
@@ -13922,13 +13927,13 @@
         <v>51</v>
       </c>
       <c r="C65" s="19" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D65" s="19" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="E65" s="19" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="F65" s="17" t="s">
         <v>16</v>
@@ -13946,7 +13951,7 @@
         <v>0</v>
       </c>
       <c r="K65" s="19" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="L65" s="19"/>
     </row>
@@ -13958,13 +13963,13 @@
         <v>51</v>
       </c>
       <c r="C66" s="19" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D66" s="19" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="E66" s="19" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F66" s="17" t="s">
         <v>16</v>
@@ -13982,7 +13987,7 @@
         <v>0</v>
       </c>
       <c r="K66" s="19" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="L66" s="19"/>
     </row>
@@ -13994,13 +13999,13 @@
         <v>51</v>
       </c>
       <c r="C67" s="19" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D67" s="19" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="E67" s="19" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="F67" s="17" t="s">
         <v>16</v>
@@ -14018,7 +14023,7 @@
         <v>0</v>
       </c>
       <c r="K67" s="19" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="L67" s="19"/>
     </row>
@@ -14030,13 +14035,13 @@
         <v>51</v>
       </c>
       <c r="C68" s="19" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D68" s="19" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E68" s="19" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F68" s="17" t="s">
         <v>16</v>
@@ -14066,13 +14071,13 @@
         <v>53</v>
       </c>
       <c r="C69" s="19" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D69" s="19" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="E69" s="19" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="F69" s="17" t="s">
         <v>16</v>
@@ -14090,7 +14095,7 @@
         <v>0</v>
       </c>
       <c r="K69" s="19" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="L69" s="19"/>
     </row>
@@ -14102,13 +14107,13 @@
         <v>53</v>
       </c>
       <c r="C70" s="19" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D70" s="19" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="E70" s="19" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="F70" s="17" t="s">
         <v>16</v>
@@ -14126,7 +14131,7 @@
         <v>0</v>
       </c>
       <c r="K70" s="19" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="L70" s="19"/>
     </row>
@@ -14138,13 +14143,13 @@
         <v>53</v>
       </c>
       <c r="C71" s="19" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D71" s="19" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E71" s="19" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="F71" s="17" t="s">
         <v>17</v>
@@ -14162,7 +14167,7 @@
         <v>0</v>
       </c>
       <c r="K71" s="19" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="L71" s="19"/>
     </row>
@@ -14174,7 +14179,7 @@
         <v>53</v>
       </c>
       <c r="C72" s="19" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D72" s="19" t="s">
         <v>264</v>
@@ -14198,7 +14203,7 @@
         <v>0</v>
       </c>
       <c r="K72" s="19" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L72" s="19"/>
     </row>
@@ -14210,13 +14215,13 @@
         <v>53</v>
       </c>
       <c r="C73" s="19" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D73" s="19" t="s">
         <v>268</v>
       </c>
       <c r="E73" s="19" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="F73" s="17" t="s">
         <v>17</v>
@@ -14234,7 +14239,7 @@
         <v>0</v>
       </c>
       <c r="K73" s="19" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="L73" s="19"/>
     </row>
@@ -14246,13 +14251,13 @@
         <v>53</v>
       </c>
       <c r="C74" s="19" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D74" s="19" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="E74" s="19" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="F74" s="17" t="s">
         <v>16</v>
@@ -14270,7 +14275,7 @@
         <v>0</v>
       </c>
       <c r="K74" s="19" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="L74" s="19"/>
     </row>
@@ -14282,13 +14287,13 @@
         <v>55</v>
       </c>
       <c r="C75" s="19" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="D75" s="19" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="E75" s="19" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="F75" s="17" t="s">
         <v>17</v>
@@ -14306,7 +14311,7 @@
         <v>0</v>
       </c>
       <c r="K75" s="19" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="L75" s="19"/>
     </row>
@@ -14318,13 +14323,13 @@
         <v>55</v>
       </c>
       <c r="C76" s="19" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="D76" s="19" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="E76" s="19" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="F76" s="17" t="s">
         <v>16</v>
@@ -14342,7 +14347,7 @@
         <v>0</v>
       </c>
       <c r="K76" s="19" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="L76" s="19"/>
     </row>
@@ -14354,13 +14359,13 @@
         <v>55</v>
       </c>
       <c r="C77" s="19" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="D77" s="19" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E77" s="19" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="F77" s="17" t="s">
         <v>16</v>
@@ -14378,7 +14383,7 @@
         <v>0</v>
       </c>
       <c r="K77" s="19" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="L77" s="19"/>
     </row>
@@ -14390,13 +14395,13 @@
         <v>55</v>
       </c>
       <c r="C78" s="19" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="D78" s="19" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E78" s="19" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="F78" s="17" t="s">
         <v>16</v>
@@ -14426,13 +14431,13 @@
         <v>55</v>
       </c>
       <c r="C79" s="19" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="D79" s="19" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="E79" s="19" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="F79" s="17" t="s">
         <v>16</v>
@@ -14450,7 +14455,7 @@
         <v>0</v>
       </c>
       <c r="K79" s="19" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="L79" s="19"/>
     </row>
@@ -14462,13 +14467,13 @@
         <v>57</v>
       </c>
       <c r="C80" s="19" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D80" s="19" t="s">
         <v>288</v>
       </c>
       <c r="E80" s="19" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="F80" s="17" t="s">
         <v>16</v>
@@ -14486,7 +14491,7 @@
         <v>0</v>
       </c>
       <c r="K80" s="19" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="L80" s="19"/>
     </row>
@@ -14498,13 +14503,13 @@
         <v>57</v>
       </c>
       <c r="C81" s="19" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D81" s="19" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E81" s="19" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="F81" s="17" t="s">
         <v>16</v>
@@ -14522,7 +14527,7 @@
         <v>0</v>
       </c>
       <c r="K81" s="19" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="L81" s="19"/>
     </row>
@@ -14534,13 +14539,13 @@
         <v>57</v>
       </c>
       <c r="C82" s="19" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D82" s="19" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="E82" s="19" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="F82" s="17" t="s">
         <v>16</v>
@@ -14558,7 +14563,7 @@
         <v>0</v>
       </c>
       <c r="K82" s="19" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="L82" s="19"/>
     </row>
@@ -14570,13 +14575,13 @@
         <v>57</v>
       </c>
       <c r="C83" s="19" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D83" s="19" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="E83" s="19" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="F83" s="17" t="s">
         <v>17</v>
@@ -14594,7 +14599,7 @@
         <v>0</v>
       </c>
       <c r="K83" s="19" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="L83" s="19"/>
     </row>
@@ -14606,13 +14611,13 @@
         <v>57</v>
       </c>
       <c r="C84" s="19" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D84" s="19" t="s">
         <v>304</v>
       </c>
       <c r="E84" s="19" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="F84" s="17" t="s">
         <v>17</v>
@@ -14630,7 +14635,7 @@
         <v>0</v>
       </c>
       <c r="K84" s="19" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="L84" s="19"/>
     </row>
@@ -14642,13 +14647,13 @@
         <v>57</v>
       </c>
       <c r="C85" s="19" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D85" s="19" t="s">
         <v>307</v>
       </c>
       <c r="E85" s="19" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="F85" s="17" t="s">
         <v>16</v>
@@ -14666,7 +14671,7 @@
         <v>0</v>
       </c>
       <c r="K85" s="19" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="L85" s="19"/>
     </row>
@@ -14678,13 +14683,13 @@
         <v>57</v>
       </c>
       <c r="C86" s="19" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D86" s="19" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="E86" s="19" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F86" s="17" t="s">
         <v>17</v>
@@ -14702,7 +14707,7 @@
         <v>0</v>
       </c>
       <c r="K86" s="19" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="L86" s="19"/>
     </row>
@@ -15688,17 +15693,17 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
     </row>
     <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15707,33 +15712,33 @@
         <v>59</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>20</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B6" s="24"/>
       <c r="C6" s="24"/>
@@ -15749,28 +15754,28 @@
         <v>1</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H7" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I7" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I7" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="8" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15778,28 +15783,28 @@
         <v>2</v>
       </c>
       <c r="B8" s="19" t="s">
+        <v>629</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>630</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>631</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>632</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>627</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>627</v>
+      </c>
+      <c r="H8" s="17" t="s">
         <v>628</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>629</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>630</v>
-      </c>
-      <c r="E8" s="25" t="s">
-        <v>631</v>
-      </c>
-      <c r="F8" s="26" t="s">
-        <v>626</v>
-      </c>
-      <c r="G8" s="17" t="s">
-        <v>626</v>
-      </c>
-      <c r="H8" s="17" t="s">
+      <c r="I8" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I8" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="9" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15807,28 +15812,28 @@
         <v>3</v>
       </c>
       <c r="B9" s="19" t="s">
+        <v>629</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>633</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>634</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>635</v>
+      </c>
+      <c r="F9" s="26" t="s">
+        <v>627</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>627</v>
+      </c>
+      <c r="H9" s="17" t="s">
         <v>628</v>
       </c>
-      <c r="C9" s="18" t="s">
-        <v>632</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>633</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>634</v>
-      </c>
-      <c r="F9" s="26" t="s">
-        <v>626</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>626</v>
-      </c>
-      <c r="H9" s="17" t="s">
+      <c r="I9" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I9" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="10" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15836,28 +15841,28 @@
         <v>4</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H10" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I10" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I10" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="11" ht="72.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15865,28 +15870,28 @@
         <v>5</v>
       </c>
       <c r="B11" s="19" t="s">
+        <v>629</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>640</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>641</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>642</v>
+      </c>
+      <c r="F11" s="26" t="s">
+        <v>627</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>627</v>
+      </c>
+      <c r="H11" s="17" t="s">
         <v>628</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>639</v>
-      </c>
-      <c r="D11" s="19" t="s">
-        <v>640</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>641</v>
-      </c>
-      <c r="F11" s="26" t="s">
-        <v>626</v>
-      </c>
-      <c r="G11" s="17" t="s">
-        <v>626</v>
-      </c>
-      <c r="H11" s="17" t="s">
+      <c r="I11" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I11" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="12" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15894,28 +15899,28 @@
         <v>6</v>
       </c>
       <c r="B12" s="19" t="s">
+        <v>629</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>643</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>644</v>
+      </c>
+      <c r="E12" s="19" t="s">
+        <v>642</v>
+      </c>
+      <c r="F12" s="26" t="s">
+        <v>627</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>627</v>
+      </c>
+      <c r="H12" s="17" t="s">
         <v>628</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>642</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>643</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>641</v>
-      </c>
-      <c r="F12" s="26" t="s">
-        <v>626</v>
-      </c>
-      <c r="G12" s="17" t="s">
-        <v>626</v>
-      </c>
-      <c r="H12" s="17" t="s">
+      <c r="I12" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I12" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="13" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15923,28 +15928,28 @@
         <v>7</v>
       </c>
       <c r="B13" s="19" t="s">
+        <v>629</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>645</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>646</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>647</v>
+      </c>
+      <c r="F13" s="26" t="s">
+        <v>627</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>627</v>
+      </c>
+      <c r="H13" s="17" t="s">
         <v>628</v>
       </c>
-      <c r="C13" s="18" t="s">
-        <v>644</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>645</v>
-      </c>
-      <c r="E13" s="25" t="s">
-        <v>646</v>
-      </c>
-      <c r="F13" s="26" t="s">
-        <v>626</v>
-      </c>
-      <c r="G13" s="17" t="s">
-        <v>626</v>
-      </c>
-      <c r="H13" s="17" t="s">
+      <c r="I13" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I13" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="14" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15952,28 +15957,28 @@
         <v>8</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="F14" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H14" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I14" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I14" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="15" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15981,28 +15986,28 @@
         <v>9</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="E15" s="25" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H15" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I15" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I15" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="16" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16010,28 +16015,28 @@
         <v>10</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="E16" s="25" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H16" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I16" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I16" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="17" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16042,25 +16047,25 @@
         <v>200</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="E17" s="25" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="F17" s="26" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H17" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I17" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I17" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="18" ht="396.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16071,25 +16076,25 @@
         <v>200</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="F18" s="26" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H18" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I18" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I18" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="19" ht="396.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16097,28 +16102,28 @@
         <v>13</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="F19" s="26" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H19" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I19" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I19" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="20" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16126,28 +16131,28 @@
         <v>14</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="F20" s="26" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H20" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I20" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I20" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="21" ht="85.4" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16155,28 +16160,28 @@
         <v>15</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="F21" s="26" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H21" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I21" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I21" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="22" ht="72.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16187,25 +16192,25 @@
         <v>217</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="F22" s="26" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H22" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I22" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I22" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="23" ht="111.2" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16213,28 +16218,28 @@
         <v>17</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="F23" s="26" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H23" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I23" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I23" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="24" ht="59.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16242,34 +16247,34 @@
         <v>18</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H24" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="I24" s="19" t="s">
         <v>627</v>
-      </c>
-      <c r="I24" s="19" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="25" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="27" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="27"/>
@@ -16288,25 +16293,25 @@
         <v>217</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="E27" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F27" s="26" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="G27" s="28" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="H27" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I27" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="28" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16317,25 +16322,25 @@
         <v>217</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E28" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F28" s="26" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="G28" s="28" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="H28" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I28" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="29" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16346,25 +16351,25 @@
         <v>217</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="E29" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F29" s="26" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="G29" s="29" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I29" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="30" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16375,25 +16380,25 @@
         <v>217</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="E30" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F30" s="26" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="G30" s="29" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="H30" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I30" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="31" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16404,25 +16409,25 @@
         <v>217</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="E31" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F31" s="26" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="G31" s="29" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="H31" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I31" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="32" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16433,25 +16438,25 @@
         <v>217</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="E32" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F32" s="26" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="G32" s="29" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="H32" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I32" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="33" ht="59.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16462,25 +16467,25 @@
         <v>217</v>
       </c>
       <c r="C33" s="18" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="E33" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F33" s="26" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="G33" s="29" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="H33" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I33" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="34" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16488,28 +16493,28 @@
         <v>26</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="E34" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F34" s="26" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="G34" s="29" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="H34" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I34" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="35" ht="111.2" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16517,28 +16522,28 @@
         <v>27</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F35" s="26" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="G35" s="28" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="H35" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I35" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="36" ht="59.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16546,28 +16551,28 @@
         <v>28</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C36" s="18" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="E36" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F36" s="26" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="G36" s="28" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="H36" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I36" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="37" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16578,25 +16583,25 @@
         <v>200</v>
       </c>
       <c r="C37" s="18" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F37" s="26" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="G37" s="28" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="H37" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I37" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16604,28 +16609,28 @@
         <v>30</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="E38" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F38" s="26" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="G38" s="29" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="H38" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I38" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="39" ht="72.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16633,28 +16638,28 @@
         <v>31</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C39" s="18" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="E39" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F39" s="26" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="G39" s="28" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="H39" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I39" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="40" ht="72.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16662,28 +16667,28 @@
         <v>32</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C40" s="18" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="E40" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F40" s="26" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="G40" s="28" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="H40" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I40" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="41" ht="59.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16691,28 +16696,28 @@
         <v>33</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C41" s="18" t="s">
         <v>154</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="E41" s="19" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="F41" s="26" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="G41" s="28" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="H41" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I41" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="42" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16720,34 +16725,34 @@
         <v>34</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C42" s="18" t="s">
         <v>326</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="E42" s="19" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="F42" s="26" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="G42" s="28" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="H42" s="17" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="I42" s="19" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="43" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="44" ht="62" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="30" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B44" s="30"/>
       <c r="C44" s="30"/>

</xml_diff>

<commit_message>
2.3.0 - rehab exercise player: programmes, sessions, check-ins, content admin
Mobile tender 2.7. Backend: RehabProgram / Block / Movement / Plan /
Session (scripts/add_rehab_program_tables.sql, applied on MnCardio_test,
with DRAFT programmes from the rehab xlsx), target heart rate at session
start, CR10 check-ins, symptom checklist on stop; /api/patient/rehab/today,
sessions, checkins; /api/doctor rehab programs and plan; /api/Media movement
and block media. Web: /admin/RehabContent. API.md §2.7c.

The Flutter screens are on branch feat/rehab-player.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/МнКардио_тендерийн_ажлын_жагсаалт.xlsx
+++ b/МнКардио_тендерийн_ажлын_жагсаалт.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2130" uniqueCount="749">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2131" uniqueCount="750">
   <si>
     <t>ХЯНАЛТЫН САМБАР</t>
   </si>
@@ -1465,7 +1465,7 @@
     <t>Дасгал үзэх, гүйцэтгэлээ тэмдэглэх боломжтой</t>
   </si>
   <si>
-    <t>2026-09-10: Энэ дэлгэцийг тэжээх сервер тал бэлэн — GET /api/patient/rehab/exercises, /rehab/progress, /rehab/vitals (веб жагсаалтын мөр #129). Гар утасны апп-ын код бичигдээгүй тул гүйцэтгэл 0 хэвээр.</t>
+    <t>2026-09-10: Энэ дэлгэцийг тэжээх сервер тал бэлэн — GET /api/patient/rehab/exercises, /rehab/progress, /rehab/vitals (веб жагсаалтын мөр #129). Гар утасны апп-ын код бичигдээгүй тул гүйцэтгэл 0 хэвээр. | 2026-09-17: Дасгалын тоглуулагч бичигдэв (сонголтын хуудсаар шийдсэн хэлбэрээр) — сервер: /api/patient/rehab/today, /sessions, /checkins (backend a88b962, API.md §2.7c), MnCardio_test-д хүснэгт ба ТӨСӨЛ хөтөлбөр (add_rehab_program_tables.sql, seed_rehab_programs_draft.sql); апп: features/rehab/rehab_today_tab, rehab_player_screen, rehab_session_summary (mncardio-github feat/rehab-player 1a4b0ee). Үлдсэн: тест сервер дээр байршуулах, APK, хөтөлбөрийн агуулгыг эмнэлзүйн баг батлах.</t>
   </si>
   <si>
     <t>Телемедицин</t>
@@ -1585,6 +1585,9 @@
     <t>Зөвлөгөө, анхааруулга харагдана</t>
   </si>
   <si>
+    <t>2026-09-17: Дасгалын өмнөх зорилтот пульсын анхааруулга (RehabProgram.WarningTemplate), 2 минут тутмын пульсын өнгөт бүс, "Биеийн байдал муу байна" шинж тэмдгийн жагсаалт + 103 сануулга — rehab_player_screen.dart. Эцсийн үг хэллэгийг сэргээн засах эмч нар батлах.</t>
+  </si>
+  <si>
     <t>39 дасгалын видео бичлэг</t>
   </si>
   <si>
@@ -1618,7 +1621,7 @@
     <t>39 анимейшн бэлэн, чанарын шаардлага хангасан</t>
   </si>
   <si>
-    <t>Анимейшн хийх зардал тендерийн үнэд багтсан | 2026-09-09: Видео бичлэг хийгдээгүй тул анимейшн эхлэх боломжгүй (захидлын 9-р зүйл).</t>
+    <t>Анимейшн хийх зардал тендерийн үнэд багтсан | 2026-09-09: Видео бичлэг хийгдээгүй тул анимейшн эхлэх боломжгүй (захидлын 9-р зүйл). | 2026-09-17: Анимейшн хийх заавар, Higgsfield prompt, бичлэгийн шаардлага (9:16, 720×1280, 3–8 сек давтагдах) бэлэн — video/higgsfield-exercise-loops.md.</t>
   </si>
   <si>
     <t>Дасгалыг апп-д байршуулах</t>
@@ -1630,7 +1633,7 @@
     <t>Дасгалууд апп дотроос үзэгдэнэ</t>
   </si>
   <si>
-    <t>2026-09-09: Видео байршуулах, хүргэх шийдэл тодорхойгүй (захидлын 10-р зүйл).</t>
+    <t>2026-09-09: Видео байршуулах, хүргэх шийдэл тодорхойгүй (захидлын 10-р зүйл). | 2026-09-17: Апп-ын талд хөдөлгөөн бүрийн давтагдах бичлэг тоглуулах, урьдчилан татах, веб админд байршуулах (/admin/RehabContent, frontend 03cde63) бэлэн. Видео ирмэгц MediaRef-д холбоно.</t>
   </si>
   <si>
     <t>Админ, тайлан</t>
@@ -11638,7 +11641,7 @@
     <col min="13" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>38</v>
       </c>
@@ -13209,10 +13212,10 @@
         <v>46263</v>
       </c>
       <c r="I45" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J45" s="23">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K45" s="19" t="s">
         <v>480</v>
@@ -13613,15 +13616,17 @@
         <v>46272</v>
       </c>
       <c r="I56" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J56" s="23">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K56" s="19" t="s">
         <v>520</v>
       </c>
-      <c r="L56" s="19"/>
+      <c r="L56" s="19" t="s">
+        <v>521</v>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="17">
@@ -13634,10 +13639,10 @@
         <v>509</v>
       </c>
       <c r="D57" s="19" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E57" s="19" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F57" s="17" t="s">
         <v>16</v>
@@ -13655,10 +13660,10 @@
         <v>0</v>
       </c>
       <c r="K57" s="19" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="L57" s="19" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -13672,10 +13677,10 @@
         <v>509</v>
       </c>
       <c r="D58" s="19" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E58" s="19" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="F58" s="17" t="s">
         <v>17</v>
@@ -13693,10 +13698,10 @@
         <v>0</v>
       </c>
       <c r="K58" s="19" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="L58" s="19" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -13710,10 +13715,10 @@
         <v>509</v>
       </c>
       <c r="D59" s="19" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E59" s="19" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="F59" s="17" t="s">
         <v>16</v>
@@ -13731,10 +13736,10 @@
         <v>0</v>
       </c>
       <c r="K59" s="19" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="L59" s="19" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -13748,10 +13753,10 @@
         <v>509</v>
       </c>
       <c r="D60" s="19" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E60" s="19" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F60" s="17" t="s">
         <v>16</v>
@@ -13769,10 +13774,10 @@
         <v>0</v>
       </c>
       <c r="K60" s="19" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="L60" s="19" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -13783,13 +13788,13 @@
         <v>51</v>
       </c>
       <c r="C61" s="19" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="D61" s="19" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="E61" s="19" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F61" s="17" t="s">
         <v>16</v>
@@ -13807,7 +13812,7 @@
         <v>0</v>
       </c>
       <c r="K61" s="19" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="L61" s="19"/>
     </row>
@@ -13819,13 +13824,13 @@
         <v>51</v>
       </c>
       <c r="C62" s="19" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="D62" s="19" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E62" s="19" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F62" s="17" t="s">
         <v>16</v>
@@ -13843,7 +13848,7 @@
         <v>0</v>
       </c>
       <c r="K62" s="19" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="L62" s="19"/>
     </row>
@@ -13855,13 +13860,13 @@
         <v>51</v>
       </c>
       <c r="C63" s="19" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="D63" s="19" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E63" s="19" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="F63" s="17" t="s">
         <v>17</v>
@@ -13879,7 +13884,7 @@
         <v>0</v>
       </c>
       <c r="K63" s="19" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="L63" s="19"/>
     </row>
@@ -13891,13 +13896,13 @@
         <v>51</v>
       </c>
       <c r="C64" s="19" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="D64" s="19" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="E64" s="19" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="F64" s="17" t="s">
         <v>16</v>
@@ -13915,7 +13920,7 @@
         <v>0</v>
       </c>
       <c r="K64" s="19" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="L64" s="19"/>
     </row>
@@ -13927,13 +13932,13 @@
         <v>51</v>
       </c>
       <c r="C65" s="19" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="D65" s="19" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E65" s="19" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="F65" s="17" t="s">
         <v>16</v>
@@ -13951,7 +13956,7 @@
         <v>0</v>
       </c>
       <c r="K65" s="19" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="L65" s="19"/>
     </row>
@@ -13963,13 +13968,13 @@
         <v>51</v>
       </c>
       <c r="C66" s="19" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="D66" s="19" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="E66" s="19" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="F66" s="17" t="s">
         <v>16</v>
@@ -13987,7 +13992,7 @@
         <v>0</v>
       </c>
       <c r="K66" s="19" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="L66" s="19"/>
     </row>
@@ -13999,13 +14004,13 @@
         <v>51</v>
       </c>
       <c r="C67" s="19" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="D67" s="19" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="E67" s="19" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F67" s="17" t="s">
         <v>16</v>
@@ -14023,7 +14028,7 @@
         <v>0</v>
       </c>
       <c r="K67" s="19" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="L67" s="19"/>
     </row>
@@ -14035,13 +14040,13 @@
         <v>51</v>
       </c>
       <c r="C68" s="19" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="D68" s="19" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="E68" s="19" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="F68" s="17" t="s">
         <v>16</v>
@@ -14071,13 +14076,13 @@
         <v>53</v>
       </c>
       <c r="C69" s="19" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D69" s="19" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="E69" s="19" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="F69" s="17" t="s">
         <v>16</v>
@@ -14095,7 +14100,7 @@
         <v>0</v>
       </c>
       <c r="K69" s="19" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="L69" s="19"/>
     </row>
@@ -14107,13 +14112,13 @@
         <v>53</v>
       </c>
       <c r="C70" s="19" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D70" s="19" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E70" s="19" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="F70" s="17" t="s">
         <v>16</v>
@@ -14131,7 +14136,7 @@
         <v>0</v>
       </c>
       <c r="K70" s="19" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="L70" s="19"/>
     </row>
@@ -14143,13 +14148,13 @@
         <v>53</v>
       </c>
       <c r="C71" s="19" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D71" s="19" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="E71" s="19" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="F71" s="17" t="s">
         <v>17</v>
@@ -14167,7 +14172,7 @@
         <v>0</v>
       </c>
       <c r="K71" s="19" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L71" s="19"/>
     </row>
@@ -14179,7 +14184,7 @@
         <v>53</v>
       </c>
       <c r="C72" s="19" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D72" s="19" t="s">
         <v>264</v>
@@ -14203,7 +14208,7 @@
         <v>0</v>
       </c>
       <c r="K72" s="19" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="L72" s="19"/>
     </row>
@@ -14215,13 +14220,13 @@
         <v>53</v>
       </c>
       <c r="C73" s="19" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D73" s="19" t="s">
         <v>268</v>
       </c>
       <c r="E73" s="19" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="F73" s="17" t="s">
         <v>17</v>
@@ -14239,7 +14244,7 @@
         <v>0</v>
       </c>
       <c r="K73" s="19" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="L73" s="19"/>
     </row>
@@ -14251,13 +14256,13 @@
         <v>53</v>
       </c>
       <c r="C74" s="19" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D74" s="19" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E74" s="19" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="F74" s="17" t="s">
         <v>16</v>
@@ -14275,7 +14280,7 @@
         <v>0</v>
       </c>
       <c r="K74" s="19" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="L74" s="19"/>
     </row>
@@ -14287,13 +14292,13 @@
         <v>55</v>
       </c>
       <c r="C75" s="19" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D75" s="19" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E75" s="19" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="F75" s="17" t="s">
         <v>17</v>
@@ -14311,7 +14316,7 @@
         <v>0</v>
       </c>
       <c r="K75" s="19" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="L75" s="19"/>
     </row>
@@ -14323,13 +14328,13 @@
         <v>55</v>
       </c>
       <c r="C76" s="19" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D76" s="19" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E76" s="19" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="F76" s="17" t="s">
         <v>16</v>
@@ -14347,7 +14352,7 @@
         <v>0</v>
       </c>
       <c r="K76" s="19" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="L76" s="19"/>
     </row>
@@ -14359,13 +14364,13 @@
         <v>55</v>
       </c>
       <c r="C77" s="19" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D77" s="19" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="E77" s="19" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="F77" s="17" t="s">
         <v>16</v>
@@ -14383,7 +14388,7 @@
         <v>0</v>
       </c>
       <c r="K77" s="19" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="L77" s="19"/>
     </row>
@@ -14395,13 +14400,13 @@
         <v>55</v>
       </c>
       <c r="C78" s="19" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D78" s="19" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="E78" s="19" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="F78" s="17" t="s">
         <v>16</v>
@@ -14431,13 +14436,13 @@
         <v>55</v>
       </c>
       <c r="C79" s="19" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D79" s="19" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="E79" s="19" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F79" s="17" t="s">
         <v>16</v>
@@ -14455,7 +14460,7 @@
         <v>0</v>
       </c>
       <c r="K79" s="19" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="L79" s="19"/>
     </row>
@@ -14467,13 +14472,13 @@
         <v>57</v>
       </c>
       <c r="C80" s="19" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="D80" s="19" t="s">
         <v>288</v>
       </c>
       <c r="E80" s="19" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="F80" s="17" t="s">
         <v>16</v>
@@ -14491,7 +14496,7 @@
         <v>0</v>
       </c>
       <c r="K80" s="19" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="L80" s="19"/>
     </row>
@@ -14503,13 +14508,13 @@
         <v>57</v>
       </c>
       <c r="C81" s="19" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="D81" s="19" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="E81" s="19" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="F81" s="17" t="s">
         <v>16</v>
@@ -14527,7 +14532,7 @@
         <v>0</v>
       </c>
       <c r="K81" s="19" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="L81" s="19"/>
     </row>
@@ -14539,13 +14544,13 @@
         <v>57</v>
       </c>
       <c r="C82" s="19" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="D82" s="19" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E82" s="19" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="F82" s="17" t="s">
         <v>16</v>
@@ -14563,7 +14568,7 @@
         <v>0</v>
       </c>
       <c r="K82" s="19" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="L82" s="19"/>
     </row>
@@ -14575,13 +14580,13 @@
         <v>57</v>
       </c>
       <c r="C83" s="19" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="D83" s="19" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E83" s="19" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="F83" s="17" t="s">
         <v>17</v>
@@ -14599,7 +14604,7 @@
         <v>0</v>
       </c>
       <c r="K83" s="19" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="L83" s="19"/>
     </row>
@@ -14611,13 +14616,13 @@
         <v>57</v>
       </c>
       <c r="C84" s="19" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="D84" s="19" t="s">
         <v>304</v>
       </c>
       <c r="E84" s="19" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="F84" s="17" t="s">
         <v>17</v>
@@ -14635,7 +14640,7 @@
         <v>0</v>
       </c>
       <c r="K84" s="19" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="L84" s="19"/>
     </row>
@@ -14647,13 +14652,13 @@
         <v>57</v>
       </c>
       <c r="C85" s="19" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="D85" s="19" t="s">
         <v>307</v>
       </c>
       <c r="E85" s="19" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="F85" s="17" t="s">
         <v>16</v>
@@ -14671,7 +14676,7 @@
         <v>0</v>
       </c>
       <c r="K85" s="19" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="L85" s="19"/>
     </row>
@@ -14683,13 +14688,13 @@
         <v>57</v>
       </c>
       <c r="C86" s="19" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="D86" s="19" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E86" s="19" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="F86" s="17" t="s">
         <v>17</v>
@@ -14707,7 +14712,7 @@
         <v>0</v>
       </c>
       <c r="K86" s="19" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="L86" s="19"/>
     </row>
@@ -15693,17 +15698,17 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15712,33 +15717,33 @@
         <v>59</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>20</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B6" s="24"/>
       <c r="C6" s="24"/>
@@ -15754,28 +15759,28 @@
         <v>1</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H7" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I7" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I7" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="8" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15783,28 +15788,28 @@
         <v>2</v>
       </c>
       <c r="B8" s="19" t="s">
+        <v>630</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>631</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>632</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>633</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>628</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="H8" s="17" t="s">
         <v>629</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>630</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>631</v>
-      </c>
-      <c r="E8" s="25" t="s">
-        <v>632</v>
-      </c>
-      <c r="F8" s="26" t="s">
-        <v>627</v>
-      </c>
-      <c r="G8" s="17" t="s">
-        <v>627</v>
-      </c>
-      <c r="H8" s="17" t="s">
+      <c r="I8" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I8" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="9" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15812,28 +15817,28 @@
         <v>3</v>
       </c>
       <c r="B9" s="19" t="s">
+        <v>630</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>634</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>635</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>636</v>
+      </c>
+      <c r="F9" s="26" t="s">
+        <v>628</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="H9" s="17" t="s">
         <v>629</v>
       </c>
-      <c r="C9" s="18" t="s">
-        <v>633</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>634</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>635</v>
-      </c>
-      <c r="F9" s="26" t="s">
-        <v>627</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>627</v>
-      </c>
-      <c r="H9" s="17" t="s">
+      <c r="I9" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I9" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="10" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15841,28 +15846,28 @@
         <v>4</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H10" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I10" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I10" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="11" ht="72.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15870,28 +15875,28 @@
         <v>5</v>
       </c>
       <c r="B11" s="19" t="s">
+        <v>630</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>641</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>642</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>643</v>
+      </c>
+      <c r="F11" s="26" t="s">
+        <v>628</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="H11" s="17" t="s">
         <v>629</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>640</v>
-      </c>
-      <c r="D11" s="19" t="s">
-        <v>641</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>642</v>
-      </c>
-      <c r="F11" s="26" t="s">
-        <v>627</v>
-      </c>
-      <c r="G11" s="17" t="s">
-        <v>627</v>
-      </c>
-      <c r="H11" s="17" t="s">
+      <c r="I11" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I11" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="12" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15899,28 +15904,28 @@
         <v>6</v>
       </c>
       <c r="B12" s="19" t="s">
+        <v>630</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>644</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>645</v>
+      </c>
+      <c r="E12" s="19" t="s">
+        <v>643</v>
+      </c>
+      <c r="F12" s="26" t="s">
+        <v>628</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="H12" s="17" t="s">
         <v>629</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>643</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>644</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>642</v>
-      </c>
-      <c r="F12" s="26" t="s">
-        <v>627</v>
-      </c>
-      <c r="G12" s="17" t="s">
-        <v>627</v>
-      </c>
-      <c r="H12" s="17" t="s">
+      <c r="I12" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I12" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="13" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15928,28 +15933,28 @@
         <v>7</v>
       </c>
       <c r="B13" s="19" t="s">
+        <v>630</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>646</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>647</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>648</v>
+      </c>
+      <c r="F13" s="26" t="s">
+        <v>628</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>628</v>
+      </c>
+      <c r="H13" s="17" t="s">
         <v>629</v>
       </c>
-      <c r="C13" s="18" t="s">
-        <v>645</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>646</v>
-      </c>
-      <c r="E13" s="25" t="s">
-        <v>647</v>
-      </c>
-      <c r="F13" s="26" t="s">
-        <v>627</v>
-      </c>
-      <c r="G13" s="17" t="s">
-        <v>627</v>
-      </c>
-      <c r="H13" s="17" t="s">
+      <c r="I13" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I13" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="14" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15957,28 +15962,28 @@
         <v>8</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="F14" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H14" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I14" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I14" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="15" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -15986,28 +15991,28 @@
         <v>9</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="E15" s="25" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H15" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I15" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I15" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="16" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16015,28 +16020,28 @@
         <v>10</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="E16" s="25" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H16" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I16" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I16" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="17" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16047,25 +16052,25 @@
         <v>200</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="E17" s="25" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="F17" s="26" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H17" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I17" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I17" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="18" ht="396.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16076,25 +16081,25 @@
         <v>200</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="F18" s="26" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H18" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I18" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I18" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="19" ht="396.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16102,28 +16107,28 @@
         <v>13</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="F19" s="26" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H19" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I19" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I19" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="20" ht="272.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16131,28 +16136,28 @@
         <v>14</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="F20" s="26" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H20" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I20" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I20" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="21" ht="85.4" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16160,28 +16165,28 @@
         <v>15</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="F21" s="26" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H21" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I21" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I21" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="22" ht="72.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16192,25 +16197,25 @@
         <v>217</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="F22" s="26" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H22" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I22" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I22" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="23" ht="111.2" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16218,28 +16223,28 @@
         <v>17</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="F23" s="26" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H23" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I23" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I23" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="24" ht="59.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16247,34 +16252,34 @@
         <v>18</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="H24" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="I24" s="19" t="s">
         <v>628</v>
-      </c>
-      <c r="I24" s="19" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="25" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="27" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="27"/>
@@ -16293,25 +16298,25 @@
         <v>217</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E27" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F27" s="26" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="G27" s="28" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="H27" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I27" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="28" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16322,25 +16327,25 @@
         <v>217</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="E28" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F28" s="26" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="G28" s="28" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="H28" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I28" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="29" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16351,25 +16356,25 @@
         <v>217</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="E29" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F29" s="26" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="G29" s="29" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I29" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="30" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16380,25 +16385,25 @@
         <v>217</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="E30" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F30" s="26" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="G30" s="29" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H30" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I30" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="31" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16409,25 +16414,25 @@
         <v>217</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="E31" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F31" s="26" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="G31" s="29" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H31" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I31" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="32" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16438,25 +16443,25 @@
         <v>217</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="E32" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F32" s="26" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="G32" s="29" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H32" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I32" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="33" ht="59.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16467,25 +16472,25 @@
         <v>217</v>
       </c>
       <c r="C33" s="18" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="E33" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F33" s="26" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="G33" s="29" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H33" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I33" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="34" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16493,28 +16498,28 @@
         <v>26</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="E34" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F34" s="26" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="G34" s="29" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H34" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I34" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="35" ht="111.2" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16522,28 +16527,28 @@
         <v>27</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="F35" s="26" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="G35" s="28" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="H35" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I35" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="36" ht="59.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16551,28 +16556,28 @@
         <v>28</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C36" s="18" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="E36" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F36" s="26" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="G36" s="28" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="H36" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I36" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="37" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16583,25 +16588,25 @@
         <v>200</v>
       </c>
       <c r="C37" s="18" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="F37" s="26" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="G37" s="28" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="H37" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I37" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="38" ht="40" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16609,28 +16614,28 @@
         <v>30</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="E38" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F38" s="26" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="G38" s="29" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H38" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I38" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="39" ht="72.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16638,28 +16643,28 @@
         <v>31</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C39" s="18" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="E39" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F39" s="26" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="G39" s="28" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="H39" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I39" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="40" ht="72.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16667,28 +16672,28 @@
         <v>32</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="C40" s="18" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="E40" s="19" t="s">
         <v>17</v>
       </c>
       <c r="F40" s="26" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="G40" s="28" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="H40" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I40" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="41" ht="59.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16696,28 +16701,28 @@
         <v>33</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="C41" s="18" t="s">
         <v>154</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="E41" s="19" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="F41" s="26" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="G41" s="28" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="H41" s="17" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I41" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="42" ht="46.7" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -16725,34 +16730,34 @@
         <v>34</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="C42" s="18" t="s">
         <v>326</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="E42" s="19" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="F42" s="26" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="G42" s="28" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="H42" s="17" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="I42" s="19" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="43" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="44" ht="62" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="30" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B44" s="30"/>
       <c r="C44" s="30"/>

</xml_diff>